<commit_message>
feat(coo): 본문 표를 No.(순번) + Customer PO로
업체가 아는 번호(Customer PO)로 읽게 한다 — CI의 PO No.와 같다.
SO Line item은 고객 PO 라인과 다른 우리 번호라 Customer PO와 짝지으면 혼란을 준다
(실측: Watergates PO WGDBS2601233을 SO 5개로 받아 DNO-2026-0020에 'PO / Line 1'이
다섯 번). 그래서 줄 번호는 1부터 순번, 정렬은 Customer PO → SO → SO 라인.
우리 SO 번호는 헤더 Order No.에 남는다.

검증: COO 테스트 54 passed, 실 DN 17건 — 맺음 블록 분할 0, 열 밀림 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/certificate_of_origin.xlsx
+++ b/templates/certificate_of_origin.xlsx
@@ -126,16 +126,16 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -588,8 +588,8 @@
   <dimension ref="A4:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -752,30 +752,30 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Order No.</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
+          <t>Customer PO</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Item No.</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>Model No. / Description</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>HS Code</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
@@ -784,15 +784,15 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>SOO-2026-0299</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
+          <t>IK29364</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>1000057706</t>
         </is>
@@ -802,7 +802,7 @@
           <t>NA015 220/240VAC-1PH-50/60HZ ALS 90-360DEG 17STAR</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>8481.90.0000</t>
         </is>

</xml_diff>